<commit_message>
docs: keep public registry detailed while reducing precision
</commit_message>
<xml_diff>
--- a/docs/catalog/FALO_Model_Dish_Registry_v0.11.xlsx
+++ b/docs/catalog/FALO_Model_Dish_Registry_v0.11.xlsx
@@ -487,7 +487,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:B17"/>
+  <dimension ref="A1:B19"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="22" customWidth="1" min="1" max="1"/>
@@ -562,7 +562,7 @@
       </c>
       <c r="B6" s="2" t="inlineStr">
         <is>
-          <t>新增 PM11、IM01-IM09、CC25、CC26；保留原版敘事密度與版本脈絡，只收斂不必要的隱私資訊。</t>
+          <t>新增 PM11、IM01-IM09、CC25、CC26；並把 Local-first IM Dev / external overview 的 Workbench 定位同步收進 IM 主線。</t>
         </is>
       </c>
     </row>
@@ -574,7 +574,7 @@
       </c>
       <c r="B7" s="2" t="inlineStr">
         <is>
-          <t>2026-05-06 21:53:03 Asia/Taipei</t>
+          <t>2026-05-06 23:35:00 Asia/Taipei</t>
         </is>
       </c>
     </row>
@@ -627,72 +627,96 @@
       </c>
     </row>
     <row r="12">
-      <c r="A12" s="2" t="inlineStr">
-        <is>
-          <t>v0.01</t>
-        </is>
-      </c>
-      <c r="B12" s="2" t="inlineStr">
-        <is>
-          <t>建立 Catalog Layer 基礎版本，整理 MM、BB、NewsOps 三大來源，並用 System / Module / Dish 做第一輪清單化。</t>
+      <c r="A12" t="inlineStr">
+        <is>
+          <t>Detail Policy</t>
+        </is>
+      </c>
+      <c r="B12" t="inlineStr">
+        <is>
+          <t>公開版與個人版都應詳細收錄各模型菜的分類與細節；公開版只降低精度，不降低內容厚度。</t>
         </is>
       </c>
     </row>
     <row r="13">
-      <c r="A13" s="2" t="inlineStr">
-        <is>
-          <t>v0.07</t>
-        </is>
-      </c>
-      <c r="B13" s="2" t="inlineStr">
-        <is>
-          <t>把母表正式化成 Excel / Markdown / HTML，統一 AA、BB、MM、CC、MMM、NewsOps 的 registry 欄位與展示格式。</t>
+      <c r="A13" t="inlineStr">
+        <is>
+          <t>Public Precision Rule</t>
+        </is>
+      </c>
+      <c r="B13" t="inlineStr">
+        <is>
+          <t>公開版保留完整分類、能力拆解、關聯與用途，但避免過度精確的敏感參數、私有路徑、環境識別與內部操作細節。</t>
         </is>
       </c>
     </row>
     <row r="14">
       <c r="A14" s="2" t="inlineStr">
         <is>
-          <t>v0.08</t>
+          <t>v0.01</t>
         </is>
       </c>
       <c r="B14" s="2" t="inlineStr">
         <is>
-          <t>將 FALO 從模型菜集合升級成 AI Task OS 導向，加入雙 NotebookLM、Skill-first、Primary / Alternative、PM / FS 主軸。</t>
+          <t>建立 Catalog Layer 基礎版本，整理 MM、BB、NewsOps 三大來源，並用 System / Module / Dish 做第一輪清單化。</t>
         </is>
       </c>
     </row>
     <row r="15">
       <c r="A15" s="2" t="inlineStr">
         <is>
-          <t>v0.09b</t>
+          <t>v0.07</t>
         </is>
       </c>
       <c r="B15" s="2" t="inlineStr">
         <is>
-          <t>將 index.html 教材頁納入 patch，新增 TEACH 系列與 PM / CC 的教學映射。</t>
+          <t>把母表正式化成 Excel / Markdown / HTML，統一 AA、BB、MM、CC、MMM、NewsOps 的 registry 欄位與展示格式。</t>
         </is>
       </c>
     </row>
     <row r="16">
       <c r="A16" s="2" t="inlineStr">
         <is>
-          <t>v0.09c</t>
+          <t>v0.08</t>
         </is>
       </c>
       <c r="B16" s="2" t="inlineStr">
         <is>
-          <t>新增 ASSET 系列，將 Sampuru AI Solution Map 登錄為 Visual Asset / AI Solution Map 型模型菜。</t>
+          <t>將 FALO 從模型菜集合升級成 AI Task OS 導向，加入雙 NotebookLM、Skill-first、Primary / Alternative、PM / FS 主軸。</t>
         </is>
       </c>
     </row>
     <row r="17">
       <c r="A17" s="2" t="inlineStr">
         <is>
+          <t>v0.09b</t>
+        </is>
+      </c>
+      <c r="B17" s="2" t="inlineStr">
+        <is>
+          <t>將 index.html 教材頁納入 patch，新增 TEACH 系列與 PM / CC 的教學映射。</t>
+        </is>
+      </c>
+    </row>
+    <row r="18">
+      <c r="A18" s="2" t="inlineStr">
+        <is>
+          <t>v0.09c</t>
+        </is>
+      </c>
+      <c r="B18" s="2" t="inlineStr">
+        <is>
+          <t>新增 ASSET 系列，將 Sampuru AI Solution Map 登錄為 Visual Asset / AI Solution Map 型模型菜。</t>
+        </is>
+      </c>
+    </row>
+    <row r="19">
+      <c r="A19" s="2" t="inlineStr">
+        <is>
           <t>v0.10</t>
         </is>
       </c>
-      <c r="B17" s="2" t="inlineStr">
+      <c r="B19" s="2" t="inlineStr">
         <is>
           <t>以 v0.09c 為基底整理發佈版，建立備份 zip 與對外寄送版本。</t>
         </is>
@@ -4242,7 +4266,7 @@
       </c>
       <c r="B6" s="3" t="inlineStr">
         <is>
-          <t>2026-05-06 21:53:03 Asia/Taipei</t>
+          <t>2026-05-06 23:35:00 Asia/Taipei</t>
         </is>
       </c>
     </row>
@@ -4546,7 +4570,7 @@
       </c>
       <c r="D2" t="inlineStr">
         <is>
-          <t>Local-first IM System</t>
+          <t>Local-first IM Workbench</t>
         </is>
       </c>
       <c r="E2" t="inlineStr">
@@ -4561,7 +4585,7 @@
       </c>
       <c r="J2" t="inlineStr">
         <is>
-          <t>Browser IM MVP</t>
+          <t>Local-first IM / AI Client Workbench</t>
         </is>
       </c>
       <c r="K2" t="inlineStr">
@@ -4571,17 +4595,17 @@
       </c>
       <c r="L2" t="inlineStr">
         <is>
-          <t>Browser client -&gt; local server -&gt; router -&gt; log -&gt; future sync</t>
+          <t>IM / room / direct message -&gt; prompt manager -&gt; export / import -&gt; GAS / Google Sheet delayed sync</t>
         </is>
       </c>
       <c r="M2" t="inlineStr">
         <is>
-          <t>Login -&gt; Join -&gt; Message -&gt; Record -&gt; Backup / Sync</t>
+          <t>Connect -&gt; Message -&gt; Prompt -&gt; Record -&gt; Export / Backup -&gt; Delayed Sync</t>
         </is>
       </c>
       <c r="N2" t="inlineStr">
         <is>
-          <t>docs/mvp/local-first-im-browser-mvp.md; apps/local-first-im/README.md; apps/local-first-im/VERSION.md</t>
+          <t>apps/local-first-im/static/index.html; apps/local-first-im/docs/external-overview.html; docs/mvp/local-first-im-browser-mvp.md; apps/local-first-im/README.md; apps/local-first-im/VERSION.md</t>
         </is>
       </c>
       <c r="O2" t="inlineStr">
@@ -4596,7 +4620,7 @@
       </c>
       <c r="Q2" t="inlineStr">
         <is>
-          <t>local-first-im, browser-client, collaboration, delayed-cloud-sync, teaching-mvp</t>
+          <t>local-first-im, ai-client-workbench, communication-os, prompt-manager, delayed-cloud-sync, gas-sync, audit-view</t>
         </is>
       </c>
       <c r="R2" t="inlineStr">
@@ -4626,17 +4650,17 @@
       </c>
       <c r="W2" t="inlineStr">
         <is>
-          <t>以地端即時、雲端延遲保存為核心的 Browser IM 系統，用來教學、測試與展示多 client 協作。</t>
+          <t>把即時通訊、AI Client、Prompt 管理與資料閉環整合在地端工作台中，作為 Falo Communication OS 的 MVP 原型。</t>
         </is>
       </c>
       <c r="X2" t="inlineStr">
         <is>
-          <t>這不是商用聊天室定稿，而是可教學、可顧問、可逐步擴充的 Local-first Collaboration System。</t>
+          <t>建議名稱可理解為 Local-first IM Workbench，也可視為 AI Client Communication Workbench。它介於 System / Module 之間，但目前以系統級模型菜原型收錄。Dev 版 index.html 偏實作介面；external-overview.html 偏外部說明版。</t>
         </is>
       </c>
       <c r="Y2" t="inlineStr">
         <is>
-          <t>Source docs: docs/mvp/local-first-im-browser-mvp.md and apps/local-first-im/*.</t>
+          <t>Sources include static/index.html as the Local-first IM Dev implementation UI and docs/external-overview.html as the external explanation page.</t>
         </is>
       </c>
       <c r="Z2" t="inlineStr">
@@ -4651,7 +4675,7 @@
       </c>
       <c r="AB2" t="inlineStr">
         <is>
-          <t>2026-05-06 21:53:03 Asia/Taipei</t>
+          <t>2026-05-06 23:05:00 Asia/Taipei</t>
         </is>
       </c>
     </row>
@@ -4673,7 +4697,7 @@
       </c>
       <c r="D3" t="inlineStr">
         <is>
-          <t>Browser Client</t>
+          <t>Local-first IM Dev Client</t>
         </is>
       </c>
       <c r="E3" t="inlineStr">
@@ -4688,7 +4712,7 @@
       </c>
       <c r="J3" t="inlineStr">
         <is>
-          <t>Web Client</t>
+          <t>Dev UI / Browser Client</t>
         </is>
       </c>
       <c r="K3" t="inlineStr">
@@ -4698,17 +4722,17 @@
       </c>
       <c r="L3" t="inlineStr">
         <is>
-          <t>Anonymous / login -&gt; room / direct message -&gt; prompt assist -&gt; copy / review</t>
+          <t>anonymous / login / address book / prompt manager / room / direct message / data loop controls</t>
         </is>
       </c>
       <c r="M3" t="inlineStr">
         <is>
-          <t>Open -&gt; Identify -&gt; Join -&gt; Send / Receive</t>
+          <t>Open -&gt; Identify -&gt; Message -&gt; Manage Prompt -&gt; Export / Import</t>
         </is>
       </c>
       <c r="N3" t="inlineStr">
         <is>
-          <t>apps/local-first-im/static/index.html; docs/mvp/local-first-im-browser-mvp.md</t>
+          <t>apps/local-first-im/static/index.html; apps/local-first-im/docs/external-overview.html</t>
         </is>
       </c>
       <c r="O3" t="inlineStr">
@@ -4718,7 +4742,7 @@
       </c>
       <c r="Q3" t="inlineStr">
         <is>
-          <t>browser-client, room-message, direct-message, prompt-copy</t>
+          <t>dev-client, browser-client, room-message, direct-message, address-book, prompt-manager, data-loop</t>
         </is>
       </c>
       <c r="R3" t="inlineStr">
@@ -4748,17 +4772,17 @@
       </c>
       <c r="W3" t="inlineStr">
         <is>
-          <t>提供人類或 AI 使用的瀏覽器介面，支援匿名進入、登入、room message、direct message 與 prompt 輔助操作。</t>
+          <t>Local-first IM Dev 實作介面版，用來測試多人、多 client、AI 角色、Prompt 管理、資料閉環與延遲同步。</t>
         </is>
       </c>
       <c r="X3" t="inlineStr">
         <is>
-          <t>教學重點是讓初學者看懂多個瀏覽器 client 如何連到同一個 local server。</t>
+          <t>這份 index.html 是 Dev 實作介面版，偏操作與測試；external-overview.html 則是對外說明版，偏非工程讀者。</t>
         </is>
       </c>
       <c r="Y3" t="inlineStr">
         <is>
-          <t>UI behavior described in docs/mvp/local-first-im-browser-mvp.md.</t>
+          <t>UI behaviors and external explanation are split between static/index.html and docs/external-overview.html.</t>
         </is>
       </c>
       <c r="Z3" t="inlineStr">
@@ -4773,7 +4797,7 @@
       </c>
       <c r="AB3" t="inlineStr">
         <is>
-          <t>2026-05-06 21:53:03 Asia/Taipei</t>
+          <t>2026-05-06 23:05:00 Asia/Taipei</t>
         </is>
       </c>
     </row>
@@ -5358,12 +5382,12 @@
       </c>
       <c r="W8" t="inlineStr">
         <is>
-          <t>提供開發測試階段的管理視角，讓使用者能查看在線狀態、全域紀錄、room 管理與備份資訊。</t>
+          <t>提供開發測試 / 稽核視角，讓使用者能查看在線狀態、全域紀錄、連線資訊、IP / session / room 狀態與備份資訊。</t>
         </is>
       </c>
       <c r="X8" t="inlineStr">
         <is>
-          <t>目前偏全員管理員視角，方便展示與測試；未來可再限縮權限。</t>
+          <t>目前偏全員管理員視角，方便展示、測試與稽核；與 Communication OS、AI Logging Shell、Local Data Hub 有高度關聯。</t>
         </is>
       </c>
       <c r="Y8" t="inlineStr">
@@ -5383,7 +5407,7 @@
       </c>
       <c r="AB8" t="inlineStr">
         <is>
-          <t>2026-05-06 21:53:03 Asia/Taipei</t>
+          <t>2026-05-06 23:05:00 Asia/Taipei</t>
         </is>
       </c>
     </row>
@@ -5480,12 +5504,12 @@
       </c>
       <c r="W9" t="inlineStr">
         <is>
-          <t>把個人 prompt 指令庫納入 IM 協作流程，支援儲存、下載、匯入與 trace 保留。</t>
+          <t>把 Prompt 新增、分類、搜尋、匯入匯出與帶入聊天室整合在個人 Prompt 管理器中。</t>
         </is>
       </c>
       <c r="X9" t="inlineStr">
         <is>
-          <t>這一模組讓 IM 不只是聊天，而是可承接 AI 指令與教學資產。</t>
+          <t>這一模組讓 IM 不只是聊天，而是可承接 AI 指令、Prompt 治理與教學資產。</t>
         </is>
       </c>
       <c r="Y9" t="inlineStr">
@@ -5505,7 +5529,7 @@
       </c>
       <c r="AB9" t="inlineStr">
         <is>
-          <t>2026-05-06 21:53:03 Asia/Taipei</t>
+          <t>2026-05-06 23:05:00 Asia/Taipei</t>
         </is>
       </c>
     </row>
@@ -5607,12 +5631,12 @@
       </c>
       <c r="W10" t="inlineStr">
         <is>
-          <t>把本地資料封裝成可備份、可追蹤、可延後同步到雲端的閉環隊列。</t>
+          <t>把 JSON / Excel 匯出匯入、本機回灌、GAS Lite 部署包與 Google Sheet 延遲同步整理成資料閉環隊列。</t>
         </is>
       </c>
       <c r="X10" t="inlineStr">
         <is>
-          <t>核心邊界是 Local-first，Cloud 延後保存；這也是這條系統最值得教的治理點之一。</t>
+          <t>核心邊界是 Local-first、Cloud delayed save；同時支援資料閉環與 GAS / Google Sheet 備份路線。</t>
         </is>
       </c>
       <c r="Y10" t="inlineStr">
@@ -5632,7 +5656,7 @@
       </c>
       <c r="AB10" t="inlineStr">
         <is>
-          <t>2026-05-06 21:53:03 Asia/Taipei</t>
+          <t>2026-05-06 23:05:00 Asia/Taipei</t>
         </is>
       </c>
     </row>
@@ -9288,7 +9312,7 @@
       </c>
       <c r="D54" t="inlineStr">
         <is>
-          <t>Local-first IM System</t>
+          <t>Local-first IM Workbench</t>
         </is>
       </c>
       <c r="E54" t="inlineStr">
@@ -9303,7 +9327,7 @@
       </c>
       <c r="J54" t="inlineStr">
         <is>
-          <t>Browser IM MVP</t>
+          <t>Local-first IM / AI Client Workbench</t>
         </is>
       </c>
       <c r="K54" t="inlineStr">
@@ -9313,17 +9337,17 @@
       </c>
       <c r="L54" t="inlineStr">
         <is>
-          <t>Browser client -&gt; local server -&gt; router -&gt; log -&gt; future sync</t>
+          <t>IM / room / direct message -&gt; prompt manager -&gt; export / import -&gt; GAS / Google Sheet delayed sync</t>
         </is>
       </c>
       <c r="M54" t="inlineStr">
         <is>
-          <t>Login -&gt; Join -&gt; Message -&gt; Record -&gt; Backup / Sync</t>
+          <t>Connect -&gt; Message -&gt; Prompt -&gt; Record -&gt; Export / Backup -&gt; Delayed Sync</t>
         </is>
       </c>
       <c r="N54" t="inlineStr">
         <is>
-          <t>docs/mvp/local-first-im-browser-mvp.md; apps/local-first-im/README.md; apps/local-first-im/VERSION.md</t>
+          <t>apps/local-first-im/static/index.html; apps/local-first-im/docs/external-overview.html; docs/mvp/local-first-im-browser-mvp.md; apps/local-first-im/README.md; apps/local-first-im/VERSION.md</t>
         </is>
       </c>
       <c r="O54" t="inlineStr">
@@ -9338,7 +9362,7 @@
       </c>
       <c r="Q54" t="inlineStr">
         <is>
-          <t>local-first-im, browser-client, collaboration, delayed-cloud-sync, teaching-mvp</t>
+          <t>local-first-im, ai-client-workbench, communication-os, prompt-manager, delayed-cloud-sync, gas-sync, audit-view</t>
         </is>
       </c>
       <c r="R54" t="inlineStr">
@@ -9368,17 +9392,17 @@
       </c>
       <c r="W54" t="inlineStr">
         <is>
-          <t>以地端即時、雲端延遲保存為核心的 Browser IM 系統，用來教學、測試與展示多 client 協作。</t>
+          <t>把即時通訊、AI Client、Prompt 管理與資料閉環整合在地端工作台中，作為 Falo Communication OS 的 MVP 原型。</t>
         </is>
       </c>
       <c r="X54" t="inlineStr">
         <is>
-          <t>這不是商用聊天室定稿，而是可教學、可顧問、可逐步擴充的 Local-first Collaboration System。</t>
+          <t>建議名稱可理解為 Local-first IM Workbench，也可視為 AI Client Communication Workbench。它介於 System / Module 之間，但目前以系統級模型菜原型收錄。Dev 版 index.html 偏實作介面；external-overview.html 偏外部說明版。</t>
         </is>
       </c>
       <c r="Y54" t="inlineStr">
         <is>
-          <t>Source docs: docs/mvp/local-first-im-browser-mvp.md and apps/local-first-im/*.</t>
+          <t>Sources include static/index.html as the Local-first IM Dev implementation UI and docs/external-overview.html as the external explanation page.</t>
         </is>
       </c>
       <c r="Z54" t="inlineStr">
@@ -9393,7 +9417,7 @@
       </c>
       <c r="AB54" t="inlineStr">
         <is>
-          <t>2026-05-06 21:53:03 Asia/Taipei</t>
+          <t>2026-05-06 23:05:00 Asia/Taipei</t>
         </is>
       </c>
     </row>
@@ -9415,7 +9439,7 @@
       </c>
       <c r="D55" t="inlineStr">
         <is>
-          <t>Browser Client</t>
+          <t>Local-first IM Dev Client</t>
         </is>
       </c>
       <c r="E55" t="inlineStr">
@@ -9430,7 +9454,7 @@
       </c>
       <c r="J55" t="inlineStr">
         <is>
-          <t>Web Client</t>
+          <t>Dev UI / Browser Client</t>
         </is>
       </c>
       <c r="K55" t="inlineStr">
@@ -9440,17 +9464,17 @@
       </c>
       <c r="L55" t="inlineStr">
         <is>
-          <t>Anonymous / login -&gt; room / direct message -&gt; prompt assist -&gt; copy / review</t>
+          <t>anonymous / login / address book / prompt manager / room / direct message / data loop controls</t>
         </is>
       </c>
       <c r="M55" t="inlineStr">
         <is>
-          <t>Open -&gt; Identify -&gt; Join -&gt; Send / Receive</t>
+          <t>Open -&gt; Identify -&gt; Message -&gt; Manage Prompt -&gt; Export / Import</t>
         </is>
       </c>
       <c r="N55" t="inlineStr">
         <is>
-          <t>apps/local-first-im/static/index.html; docs/mvp/local-first-im-browser-mvp.md</t>
+          <t>apps/local-first-im/static/index.html; apps/local-first-im/docs/external-overview.html</t>
         </is>
       </c>
       <c r="O55" t="inlineStr">
@@ -9460,7 +9484,7 @@
       </c>
       <c r="Q55" t="inlineStr">
         <is>
-          <t>browser-client, room-message, direct-message, prompt-copy</t>
+          <t>dev-client, browser-client, room-message, direct-message, address-book, prompt-manager, data-loop</t>
         </is>
       </c>
       <c r="R55" t="inlineStr">
@@ -9490,17 +9514,17 @@
       </c>
       <c r="W55" t="inlineStr">
         <is>
-          <t>提供人類或 AI 使用的瀏覽器介面，支援匿名進入、登入、room message、direct message 與 prompt 輔助操作。</t>
+          <t>Local-first IM Dev 實作介面版，用來測試多人、多 client、AI 角色、Prompt 管理、資料閉環與延遲同步。</t>
         </is>
       </c>
       <c r="X55" t="inlineStr">
         <is>
-          <t>教學重點是讓初學者看懂多個瀏覽器 client 如何連到同一個 local server。</t>
+          <t>這份 index.html 是 Dev 實作介面版，偏操作與測試；external-overview.html 則是對外說明版，偏非工程讀者。</t>
         </is>
       </c>
       <c r="Y55" t="inlineStr">
         <is>
-          <t>UI behavior described in docs/mvp/local-first-im-browser-mvp.md.</t>
+          <t>UI behaviors and external explanation are split between static/index.html and docs/external-overview.html.</t>
         </is>
       </c>
       <c r="Z55" t="inlineStr">
@@ -9515,7 +9539,7 @@
       </c>
       <c r="AB55" t="inlineStr">
         <is>
-          <t>2026-05-06 21:53:03 Asia/Taipei</t>
+          <t>2026-05-06 23:05:00 Asia/Taipei</t>
         </is>
       </c>
     </row>
@@ -10100,12 +10124,12 @@
       </c>
       <c r="W60" t="inlineStr">
         <is>
-          <t>提供開發測試階段的管理視角，讓使用者能查看在線狀態、全域紀錄、room 管理與備份資訊。</t>
+          <t>提供開發測試 / 稽核視角，讓使用者能查看在線狀態、全域紀錄、連線資訊、IP / session / room 狀態與備份資訊。</t>
         </is>
       </c>
       <c r="X60" t="inlineStr">
         <is>
-          <t>目前偏全員管理員視角，方便展示與測試；未來可再限縮權限。</t>
+          <t>目前偏全員管理員視角，方便展示、測試與稽核；與 Communication OS、AI Logging Shell、Local Data Hub 有高度關聯。</t>
         </is>
       </c>
       <c r="Y60" t="inlineStr">
@@ -10125,7 +10149,7 @@
       </c>
       <c r="AB60" t="inlineStr">
         <is>
-          <t>2026-05-06 21:53:03 Asia/Taipei</t>
+          <t>2026-05-06 23:05:00 Asia/Taipei</t>
         </is>
       </c>
     </row>
@@ -10222,12 +10246,12 @@
       </c>
       <c r="W61" t="inlineStr">
         <is>
-          <t>把個人 prompt 指令庫納入 IM 協作流程，支援儲存、下載、匯入與 trace 保留。</t>
+          <t>把 Prompt 新增、分類、搜尋、匯入匯出與帶入聊天室整合在個人 Prompt 管理器中。</t>
         </is>
       </c>
       <c r="X61" t="inlineStr">
         <is>
-          <t>這一模組讓 IM 不只是聊天，而是可承接 AI 指令與教學資產。</t>
+          <t>這一模組讓 IM 不只是聊天，而是可承接 AI 指令、Prompt 治理與教學資產。</t>
         </is>
       </c>
       <c r="Y61" t="inlineStr">
@@ -10247,7 +10271,7 @@
       </c>
       <c r="AB61" t="inlineStr">
         <is>
-          <t>2026-05-06 21:53:03 Asia/Taipei</t>
+          <t>2026-05-06 23:05:00 Asia/Taipei</t>
         </is>
       </c>
     </row>
@@ -10349,12 +10373,12 @@
       </c>
       <c r="W62" t="inlineStr">
         <is>
-          <t>把本地資料封裝成可備份、可追蹤、可延後同步到雲端的閉環隊列。</t>
+          <t>把 JSON / Excel 匯出匯入、本機回灌、GAS Lite 部署包與 Google Sheet 延遲同步整理成資料閉環隊列。</t>
         </is>
       </c>
       <c r="X62" t="inlineStr">
         <is>
-          <t>核心邊界是 Local-first，Cloud 延後保存；這也是這條系統最值得教的治理點之一。</t>
+          <t>核心邊界是 Local-first、Cloud delayed save；同時支援資料閉環與 GAS / Google Sheet 備份路線。</t>
         </is>
       </c>
       <c r="Y62" t="inlineStr">
@@ -10374,7 +10398,7 @@
       </c>
       <c r="AB62" t="inlineStr">
         <is>
-          <t>2026-05-06 21:53:03 Asia/Taipei</t>
+          <t>2026-05-06 23:05:00 Asia/Taipei</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
docs: align public edition as detailed readable version
</commit_message>
<xml_diff>
--- a/docs/catalog/FALO_Model_Dish_Registry_v0.11.xlsx
+++ b/docs/catalog/FALO_Model_Dish_Registry_v0.11.xlsx
@@ -574,7 +574,7 @@
       </c>
       <c r="B7" s="2" t="inlineStr">
         <is>
-          <t>2026-05-06 23:35:00 Asia/Taipei</t>
+          <t>2026-05-06 22:56:02 Asia/Taipei</t>
         </is>
       </c>
     </row>
@@ -586,7 +586,7 @@
       </c>
       <c r="B8" t="inlineStr">
         <is>
-          <t>Original-reference Privacy Edition</t>
+          <t>公開可讀的詳細版</t>
         </is>
       </c>
     </row>
@@ -4266,7 +4266,7 @@
       </c>
       <c r="B6" s="3" t="inlineStr">
         <is>
-          <t>2026-05-06 23:35:00 Asia/Taipei</t>
+          <t>2026-05-06 22:56:02 Asia/Taipei</t>
         </is>
       </c>
     </row>
@@ -4391,7 +4391,7 @@
       </c>
       <c r="B8" t="inlineStr">
         <is>
-          <t>推出高度參考原版的 GitHub-ready 隱私版，新增 PM11、IM 系列與公開版隱私邊界。</t>
+          <t>推出高度參考原版的 GitHub-ready 公開可讀詳細版，新增 PM11、IM 系列與公開版隱私邊界。</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
docs: sync workbook for im visual asset set
</commit_message>
<xml_diff>
--- a/docs/catalog/FALO_Model_Dish_Registry_v0.11.xlsx
+++ b/docs/catalog/FALO_Model_Dish_Registry_v0.11.xlsx
@@ -514,7 +514,7 @@
       </c>
       <c r="B2" s="2" t="inlineStr">
         <is>
-          <t>v0.11 original-reference privacy edition</t>
+          <t>v0.11 public detailed edition</t>
         </is>
       </c>
     </row>
@@ -562,7 +562,7 @@
       </c>
       <c r="B6" s="2" t="inlineStr">
         <is>
-          <t>新增 PM11、IM01-IM09、CC25、CC26；並把 Local-first IM Dev / external overview 的 Workbench 定位同步收進 IM 主線。</t>
+          <t>新增 PM11、IM01-IM09、CC25、CC26，並補入 ASSET02 作為 Local-first IM 的四張一組視覺說明資產。</t>
         </is>
       </c>
     </row>
@@ -718,7 +718,7 @@
       </c>
       <c r="B19" s="2" t="inlineStr">
         <is>
-          <t>以 v0.09c 為基底整理發佈版，建立備份 zip 與對外寄送版本。</t>
+          <t>2026-05-06 23:18:00 Asia/Taipei</t>
         </is>
       </c>
     </row>
@@ -1249,7 +1249,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:AB2"/>
+  <dimension ref="A1:AB3"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="12" customWidth="1" min="1" max="1"/>
@@ -1542,6 +1542,118 @@
       <c r="AB2" s="3" t="inlineStr">
         <is>
           <t>2026-05-06 00:01:59 Asia/Taipei</t>
+        </is>
+      </c>
+    </row>
+    <row r="3">
+      <c r="A3" t="inlineStr">
+        <is>
+          <t>ASSET</t>
+        </is>
+      </c>
+      <c r="B3" t="inlineStr">
+        <is>
+          <t>Visual Asset / IM Workbench Explainer Set</t>
+        </is>
+      </c>
+      <c r="C3" t="inlineStr">
+        <is>
+          <t>ASSET02</t>
+        </is>
+      </c>
+      <c r="D3" t="inlineStr">
+        <is>
+          <t>Local-first IM Workbench Visual Explainer Set</t>
+        </is>
+      </c>
+      <c r="E3" t="inlineStr">
+        <is>
+          <t>Visual Asset Set / Model Dish</t>
+        </is>
+      </c>
+      <c r="F3" t="inlineStr">
+        <is>
+          <t>Visual Storytelling / Teaching / System Explainer</t>
+        </is>
+      </c>
+      <c r="J3" t="inlineStr">
+        <is>
+          <t>Image Set</t>
+        </is>
+      </c>
+      <c r="K3" t="inlineStr">
+        <is>
+          <t>Teaching + Consulting + Showcase</t>
+        </is>
+      </c>
+      <c r="N3" t="inlineStr">
+        <is>
+          <t>ChatGPT Image 2026年5月6日 下午11_00_30.png | ChatGPT Image 2026年5月6日 下午11_00_33.png | ChatGPT Image 2026年5月6日 下午11_00_38.png | ChatGPT Image 2026年5月6日 下午11_00_41.png</t>
+        </is>
+      </c>
+      <c r="O3" t="inlineStr">
+        <is>
+          <t>private local image set (not bundled)</t>
+        </is>
+      </c>
+      <c r="Q3" t="inlineStr">
+        <is>
+          <t>local-first-im, visual-explainer, teaching-asset, system-overview, scenario-map, im-workbench, mvp-usable</t>
+        </is>
+      </c>
+      <c r="R3" t="inlineStr">
+        <is>
+          <t>v0.11</t>
+        </is>
+      </c>
+      <c r="S3" t="inlineStr">
+        <is>
+          <t>visual_asset</t>
+        </is>
+      </c>
+      <c r="T3" t="inlineStr">
+        <is>
+          <t>teaching_material</t>
+        </is>
+      </c>
+      <c r="U3" t="inlineStr">
+        <is>
+          <t>candidate</t>
+        </is>
+      </c>
+      <c r="V3" t="inlineStr">
+        <is>
+          <t>ASSET, IM, PM, TRACE</t>
+        </is>
+      </c>
+      <c r="W3" t="inlineStr">
+        <is>
+          <t>以四張單頁圖解，分別從簡單版、情境版、情境精華版與最複雜版，展示 Local-first IM Workbench 的不同敘事深度與系統切面。</t>
+        </is>
+      </c>
+      <c r="X3" t="inlineStr">
+        <is>
+          <t>這四張是一套，不應拆成四個零散條目。適合用於教學、顧問提案、系統說明與視覺導覽；同時作為 IM01 的外部展示資產。</t>
+        </is>
+      </c>
+      <c r="Y3" t="inlineStr">
+        <is>
+          <t>Includes Local-first IM MVP 簡單版, Local-first IM Workbench 情境版, 情境精華版, and 最複雜版 v0.05-dev.</t>
+        </is>
+      </c>
+      <c r="Z3" t="inlineStr">
+        <is>
+          <t>POC complete / Teaching-ready</t>
+        </is>
+      </c>
+      <c r="AA3" t="inlineStr">
+        <is>
+          <t>v0.11</t>
+        </is>
+      </c>
+      <c r="AB3" t="inlineStr">
+        <is>
+          <t>2026-05-06 23:18:00 Asia/Taipei</t>
         </is>
       </c>
     </row>
@@ -4655,12 +4767,12 @@
       </c>
       <c r="X2" t="inlineStr">
         <is>
-          <t>建議名稱可理解為 Local-first IM Workbench，也可視為 AI Client Communication Workbench。它介於 System / Module 之間，但目前以系統級模型菜原型收錄。Dev 版 index.html 偏實作介面；external-overview.html 偏外部說明版。</t>
+          <t>建議名稱可理解為 Local-first IM Workbench，也可視為 AI Client Communication Workbench。它介於 System / Module 之間，但目前以系統級模型菜原型收錄。Dev 版 index.html 偏實作介面；external-overview.html 偏外部說明版。 另有一組四張單頁視覺圖解，已收錄為 ASSET02，作為 IM01 的外部展示資產。</t>
         </is>
       </c>
       <c r="Y2" t="inlineStr">
         <is>
-          <t>Sources include static/index.html as the Local-first IM Dev implementation UI and docs/external-overview.html as the external explanation page.</t>
+          <t>Sources include static/index.html as the Local-first IM Dev implementation UI and docs/external-overview.html as the external explanation page. Visual explainer set grouped as ASSET02.</t>
         </is>
       </c>
       <c r="Z2" t="inlineStr">
@@ -4675,7 +4787,7 @@
       </c>
       <c r="AB2" t="inlineStr">
         <is>
-          <t>2026-05-06 23:05:00 Asia/Taipei</t>
+          <t>2026-05-06 23:18:00 Asia/Taipei</t>
         </is>
       </c>
     </row>
@@ -5671,7 +5783,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:AB157"/>
+  <dimension ref="A1:AB158"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="12" customWidth="1" min="1" max="1"/>
@@ -9397,12 +9509,12 @@
       </c>
       <c r="X54" t="inlineStr">
         <is>
-          <t>建議名稱可理解為 Local-first IM Workbench，也可視為 AI Client Communication Workbench。它介於 System / Module 之間，但目前以系統級模型菜原型收錄。Dev 版 index.html 偏實作介面；external-overview.html 偏外部說明版。</t>
+          <t>建議名稱可理解為 Local-first IM Workbench，也可視為 AI Client Communication Workbench。它介於 System / Module 之間，但目前以系統級模型菜原型收錄。Dev 版 index.html 偏實作介面；external-overview.html 偏外部說明版。 另有一組四張單頁視覺圖解，已收錄為 ASSET02，作為 IM01 的外部展示資產。</t>
         </is>
       </c>
       <c r="Y54" t="inlineStr">
         <is>
-          <t>Sources include static/index.html as the Local-first IM Dev implementation UI and docs/external-overview.html as the external explanation page.</t>
+          <t>Sources include static/index.html as the Local-first IM Dev implementation UI and docs/external-overview.html as the external explanation page. Visual explainer set grouped as ASSET02.</t>
         </is>
       </c>
       <c r="Z54" t="inlineStr">
@@ -9417,7 +9529,7 @@
       </c>
       <c r="AB54" t="inlineStr">
         <is>
-          <t>2026-05-06 23:05:00 Asia/Taipei</t>
+          <t>2026-05-06 23:18:00 Asia/Taipei</t>
         </is>
       </c>
     </row>
@@ -16269,6 +16381,118 @@
       <c r="AB157" t="inlineStr">
         <is>
           <t>2026-05-06 00:01:59 Asia/Taipei</t>
+        </is>
+      </c>
+    </row>
+    <row r="158">
+      <c r="A158" t="inlineStr">
+        <is>
+          <t>ASSET</t>
+        </is>
+      </c>
+      <c r="B158" t="inlineStr">
+        <is>
+          <t>Visual Asset / IM Workbench Explainer Set</t>
+        </is>
+      </c>
+      <c r="C158" t="inlineStr">
+        <is>
+          <t>ASSET02</t>
+        </is>
+      </c>
+      <c r="D158" t="inlineStr">
+        <is>
+          <t>Local-first IM Workbench Visual Explainer Set</t>
+        </is>
+      </c>
+      <c r="E158" t="inlineStr">
+        <is>
+          <t>Visual Asset Set / Model Dish</t>
+        </is>
+      </c>
+      <c r="F158" t="inlineStr">
+        <is>
+          <t>Visual Storytelling / Teaching / System Explainer</t>
+        </is>
+      </c>
+      <c r="J158" t="inlineStr">
+        <is>
+          <t>Image Set</t>
+        </is>
+      </c>
+      <c r="K158" t="inlineStr">
+        <is>
+          <t>Teaching + Consulting + Showcase</t>
+        </is>
+      </c>
+      <c r="N158" t="inlineStr">
+        <is>
+          <t>ChatGPT Image 2026年5月6日 下午11_00_30.png | ChatGPT Image 2026年5月6日 下午11_00_33.png | ChatGPT Image 2026年5月6日 下午11_00_38.png | ChatGPT Image 2026年5月6日 下午11_00_41.png</t>
+        </is>
+      </c>
+      <c r="O158" t="inlineStr">
+        <is>
+          <t>private local image set (not bundled)</t>
+        </is>
+      </c>
+      <c r="Q158" t="inlineStr">
+        <is>
+          <t>local-first-im, visual-explainer, teaching-asset, system-overview, scenario-map, im-workbench, mvp-usable</t>
+        </is>
+      </c>
+      <c r="R158" t="inlineStr">
+        <is>
+          <t>v0.11</t>
+        </is>
+      </c>
+      <c r="S158" t="inlineStr">
+        <is>
+          <t>visual_asset</t>
+        </is>
+      </c>
+      <c r="T158" t="inlineStr">
+        <is>
+          <t>teaching_material</t>
+        </is>
+      </c>
+      <c r="U158" t="inlineStr">
+        <is>
+          <t>candidate</t>
+        </is>
+      </c>
+      <c r="V158" t="inlineStr">
+        <is>
+          <t>ASSET, IM, PM, TRACE</t>
+        </is>
+      </c>
+      <c r="W158" t="inlineStr">
+        <is>
+          <t>以四張單頁圖解，分別從簡單版、情境版、情境精華版與最複雜版，展示 Local-first IM Workbench 的不同敘事深度與系統切面。</t>
+        </is>
+      </c>
+      <c r="X158" t="inlineStr">
+        <is>
+          <t>這四張是一套，不應拆成四個零散條目。適合用於教學、顧問提案、系統說明與視覺導覽；同時作為 IM01 的外部展示資產。</t>
+        </is>
+      </c>
+      <c r="Y158" t="inlineStr">
+        <is>
+          <t>Includes Local-first IM MVP 簡單版, Local-first IM Workbench 情境版, 情境精華版, and 最複雜版 v0.05-dev.</t>
+        </is>
+      </c>
+      <c r="Z158" t="inlineStr">
+        <is>
+          <t>POC complete / Teaching-ready</t>
+        </is>
+      </c>
+      <c r="AA158" t="inlineStr">
+        <is>
+          <t>v0.11</t>
+        </is>
+      </c>
+      <c r="AB158" t="inlineStr">
+        <is>
+          <t>2026-05-06 23:18:00 Asia/Taipei</t>
         </is>
       </c>
     </row>

</xml_diff>